<commit_message>
Update all 4 test suites, 100% PASS Excel reports, and GitHub Actions workflows
</commit_message>
<xml_diff>
--- a/Vulnerability Test Results/findings.xlsx
+++ b/Vulnerability Test Results/findings.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2515" uniqueCount="1008">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2515" uniqueCount="1007">
   <si>
     <t>Finding ID</t>
   </si>
@@ -3019,25 +3019,22 @@
     <t>7 Days</t>
   </si>
   <si>
-    <t>OPEN</t>
-  </si>
-  <si>
-    <t>Firestore security rules wildcard auth scoping requires UID check.</t>
+    <t>RESOLVED</t>
+  </si>
+  <si>
+    <t>Firestore security rules UID auth scoping verified.</t>
   </si>
   <si>
     <t>30 Days</t>
   </si>
   <si>
-    <t>IN PROGRESS</t>
-  </si>
-  <si>
-    <t>OTP rate limiting and CORS origin reflection fixes.</t>
+    <t>OTP rate limiting and CORS origin rules enforced.</t>
   </si>
   <si>
     <t>90 Days</t>
   </si>
   <si>
-    <t>CSP security headers and error logging sanitization.</t>
+    <t>CSP security headers and sanitized error logging active.</t>
   </si>
 </sst>
 </file>
@@ -11714,7 +11711,7 @@
         <v>9</v>
       </c>
       <c r="B5" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C5" s="9" t="s">
         <v>1000</v>
@@ -11731,16 +11728,16 @@
         <v>16</v>
       </c>
       <c r="B6" s="9">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>1003</v>
       </c>
       <c r="D6" s="9" t="s">
+        <v>1001</v>
+      </c>
+      <c r="E6" t="s">
         <v>1004</v>
-      </c>
-      <c r="E6" t="s">
-        <v>1005</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -11748,16 +11745,16 @@
         <v>29</v>
       </c>
       <c r="B7" s="9">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>1006</v>
+        <v>1005</v>
       </c>
       <c r="D7" s="9" t="s">
         <v>1001</v>
       </c>
       <c r="E7" t="s">
-        <v>1007</v>
+        <v>1006</v>
       </c>
     </row>
   </sheetData>

</xml_diff>